<commit_message>
adding safe version of ele data - just distances from water sources
</commit_message>
<xml_diff>
--- a/00_metadata/elephant_analysis_metadata.xlsx
+++ b/00_metadata/elephant_analysis_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/margaretswift/Documents/03 Science/00 Research - Active/Ecosphere Waterholes/eco-kaza-water-ele/00_metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7AB00F-2877-8041-949A-2584EE4D4B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCC9414-92EF-9940-B6EA-B45009F27123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="-7880" windowWidth="20020" windowHeight="21100" activeTab="2" xr2:uid="{36B2674D-5574-5749-ABD1-0B06D0B52360}"/>
+    <workbookView xWindow="29400" yWindow="-7880" windowWidth="20020" windowHeight="21100" activeTab="3" xr2:uid="{36B2674D-5574-5749-ABD1-0B06D0B52360}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="175">
   <si>
     <t>Column Name</t>
   </si>
@@ -277,9 +277,6 @@
     <t>02_addWaterDistsToEle.R</t>
   </si>
   <si>
-    <t>ele.dat</t>
-  </si>
-  <si>
     <t>ESW_NN_ID</t>
   </si>
   <si>
@@ -397,12 +394,6 @@
     <t>LC21_NN_RECUR</t>
   </si>
   <si>
-    <t>DATE</t>
-  </si>
-  <si>
-    <t>Date of GPS point</t>
-  </si>
-  <si>
     <t>Year of GPS point</t>
   </si>
   <si>
@@ -526,16 +517,37 @@
     <t>recurrence of nearest neighbor (KAZA 2021 landcover)</t>
   </si>
   <si>
-    <t>/01_data/elephant/processed/elephant_with_dists.rdata</t>
-  </si>
-  <si>
-    <t>Elephant GPS collar data with distance-to-water added for all water indices</t>
-  </si>
-  <si>
     <t>MFREQ</t>
   </si>
   <si>
     <t xml:space="preserve">mean frequency of nearest ESW surface water </t>
+  </si>
+  <si>
+    <t>ID (sequential) of elephant</t>
+  </si>
+  <si>
+    <t>was this the first GPS point of a new burst?</t>
+  </si>
+  <si>
+    <t>boolean</t>
+  </si>
+  <si>
+    <t>num</t>
+  </si>
+  <si>
+    <t>ele.safe.dat</t>
+  </si>
+  <si>
+    <t>Distance-to-water  for all water indices</t>
+  </si>
+  <si>
+    <t>/03_output/02_elephant_analysis/elephant_analysis.rdata</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>GPS location and date-time data have been removed for the public dataset.</t>
   </si>
 </sst>
 </file>
@@ -1041,7 +1053,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1052,32 +1064,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1500,254 +1493,253 @@
   <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="58.6640625" style="7" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="7"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="6">
         <v>86000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>7990000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="4">
         <v>3.4</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="11"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="11"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B17" s="9"/>
+      <c r="B17" s="2"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B18" s="9"/>
+      <c r="B18" s="2"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B19" s="9"/>
+      <c r="B19" s="2"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B20" s="9"/>
+      <c r="B20" s="2"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B21" s="9"/>
+      <c r="B21" s="2"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B22" s="9"/>
+      <c r="B22" s="2"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B23" s="9"/>
+      <c r="B23" s="2"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B24" s="9"/>
+      <c r="B24" s="2"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="6"/>
+      <c r="A28" s="1"/>
     </row>
     <row r="29" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="6"/>
+      <c r="A29" s="1"/>
     </row>
     <row r="30" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="6"/>
+      <c r="A30" s="1"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="6"/>
+      <c r="A31" s="1"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="8"/>
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="3"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="9"/>
-      <c r="D34" s="10"/>
+      <c r="A34" s="2"/>
+      <c r="D34" s="6"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="9"/>
-      <c r="B35" s="9"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="11"/>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="11"/>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="4"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="9"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="11"/>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="4"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="9"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="11"/>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="4"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="9"/>
-      <c r="B40" s="9"/>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="9"/>
-      <c r="B41" s="9"/>
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9"/>
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B44" s="9"/>
+      <c r="B44" s="2"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B45" s="9"/>
+      <c r="B45" s="2"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B46" s="9"/>
+      <c r="B46" s="2"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B47" s="9"/>
+      <c r="B47" s="2"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B48" s="9"/>
+      <c r="B48" s="2"/>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B49" s="9"/>
+      <c r="B49" s="2"/>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B50" s="9"/>
+      <c r="B50" s="2"/>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B51" s="9"/>
+      <c r="B51" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1759,322 +1751,321 @@
   <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="56" style="7" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="47.6640625" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="7"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="56" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="47.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="4">
         <v>1001</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="4">
         <v>860000</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="4">
         <v>7990000</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="11" t="b">
+      <c r="D12" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="4" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="4" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="4">
         <v>240</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="4">
         <v>14400</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="4">
         <v>443</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="4">
         <v>240</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="4">
         <v>-1.4</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="4">
         <v>0.51</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="4" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2085,7 +2076,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12DD8F44-6D9D-3C43-9B42-3CFE39D46E45}">
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -2094,316 +2085,306 @@
     <col min="4" max="4" width="27.83203125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="11"/>
-    </row>
-    <row r="2" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="11"/>
-    </row>
-    <row r="3" spans="1:4" s="7" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="11"/>
-    </row>
-    <row r="4" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+      <c r="C10" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D10" s="6" t="b">
         <v>1</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="D4" s="11"/>
-    </row>
-    <row r="6" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" s="11">
-        <v>1001</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="11">
-        <v>860000</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="11">
-        <v>7990000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="11" t="b">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>36</v>
+      <c r="D13" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>37</v>
+        <v>85</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1000</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>38</v>
+        <v>86</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D15" s="4">
+        <v>3.4</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>39</v>
+      <c r="D16" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="11">
-        <v>240</v>
+        <v>88</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="11">
-        <v>14400</v>
+        <v>89</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D18" s="4">
+        <v>3.4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="11">
-        <v>443</v>
+        <v>90</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="11">
-        <v>240</v>
+        <v>91</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1000</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="11">
-        <v>-1.4</v>
+        <v>92</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="4">
+        <v>3.4</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D22" s="11">
-        <v>0.51</v>
+        <v>93</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="16" t="s">
-        <v>35</v>
+        <v>94</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D24" s="4">
+        <v>3.4</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="C25" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="4">
@@ -2412,12 +2393,12 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="C26" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D26" s="4">
@@ -2426,13 +2407,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>87</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>130</v>
+        <v>98</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D27" s="4">
         <v>3.4</v>
@@ -2440,12 +2421,12 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C28" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D28" s="4">
@@ -2454,12 +2435,12 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>89</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="C29" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D29" s="4">
@@ -2468,13 +2449,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>90</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>130</v>
+        <v>101</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D30" s="4">
         <v>3.4</v>
@@ -2482,12 +2463,12 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>91</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="C31" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D31" s="4">
@@ -2496,12 +2477,12 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>92</v>
-      </c>
-      <c r="B32" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="C32" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D32" s="4">
@@ -2510,13 +2491,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>93</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>130</v>
+        <v>104</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D33" s="4">
         <v>3.4</v>
@@ -2524,12 +2505,12 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>94</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="C34" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D34" s="4">
@@ -2538,12 +2519,12 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>95</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="C35" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D35" s="4">
@@ -2552,13 +2533,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>96</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>130</v>
+        <v>107</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D36" s="4">
         <v>3.4</v>
@@ -2566,12 +2547,12 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>97</v>
-      </c>
-      <c r="B37" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C37" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D37" s="4">
@@ -2580,12 +2561,12 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>98</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="C38" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D38" s="4">
@@ -2594,13 +2575,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>99</v>
-      </c>
-      <c r="B39" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>130</v>
+        <v>110</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D39" s="4">
         <v>3.4</v>
@@ -2608,12 +2589,12 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>100</v>
-      </c>
-      <c r="B40" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="C40" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C40" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D40" s="4">
@@ -2622,12 +2603,12 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>101</v>
-      </c>
-      <c r="B41" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="C41" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D41" s="4">
@@ -2636,13 +2617,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>102</v>
-      </c>
-      <c r="B42" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>130</v>
+        <v>113</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D42" s="4">
         <v>3.4</v>
@@ -2650,12 +2631,12 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>103</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="C43" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D43" s="4">
@@ -2664,12 +2645,12 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="C44" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D44" s="4">
@@ -2678,13 +2659,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>105</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>130</v>
+        <v>116</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D45" s="4">
         <v>3.4</v>
@@ -2692,12 +2673,12 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>106</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="C46" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D46" s="4">
@@ -2706,12 +2687,12 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>107</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="C47" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C47" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D47" s="4">
@@ -2720,13 +2701,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>108</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="C48" s="15" t="s">
-        <v>130</v>
+        <v>119</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D48" s="4">
         <v>3.4</v>
@@ -2734,12 +2715,12 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>109</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="C49" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D49" s="4">
@@ -2748,12 +2729,12 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>110</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="C50" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C50" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D50" s="4">
@@ -2762,240 +2743,30 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>111</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="C51" s="15" t="s">
-        <v>130</v>
+        <v>122</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="D51" s="4">
         <v>3.4</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>112</v>
-      </c>
-      <c r="B52" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="C52" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D52" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>113</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D53" s="4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>114</v>
-      </c>
-      <c r="B54" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C54" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="D54" s="4">
+    <row r="52" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D52" s="8">
         <v>3.4</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>115</v>
-      </c>
-      <c r="B55" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="C55" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D55" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>116</v>
-      </c>
-      <c r="B56" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="C56" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D56" s="4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>117</v>
-      </c>
-      <c r="B57" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="C57" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="D57" s="4">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>118</v>
-      </c>
-      <c r="B58" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="C58" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D58" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>119</v>
-      </c>
-      <c r="B59" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="C59" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D59" s="4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>120</v>
-      </c>
-      <c r="B60" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="C60" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="D60" s="4">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>121</v>
-      </c>
-      <c r="B61" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="C61" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D61" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>122</v>
-      </c>
-      <c r="B62" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="C62" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D62" s="4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="B63" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="C63" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="D63" s="11">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B64" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="C64" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="D64" s="16">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>30</v>
-      </c>
-      <c r="B65" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="D65" s="11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>124</v>
-      </c>
-      <c r="B66" t="s">
-        <v>125</v>
-      </c>
-      <c r="C66" t="s">
-        <v>59</v>
-      </c>
-      <c r="D66" s="12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>9</v>
-      </c>
-      <c r="B67" t="s">
-        <v>126</v>
-      </c>
-      <c r="C67" t="s">
-        <v>10</v>
-      </c>
-      <c r="D67" s="4">
-        <v>2015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>